<commit_message>
made changes to some xpaths
</commit_message>
<xml_diff>
--- a/testdata/Scenario1_2_3_TestData.xlsx
+++ b/testdata/Scenario1_2_3_TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2408439\CTS_Java_Training\Practicals\IntelliJ_Selenium_Projects\Hackathon_Project\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66227E41-EE1C-451D-8198-1B8900B4E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A338126-090B-4B44-80A4-2A088B5CC373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DE57E9C9-A6C1-4A7D-85B9-1309751074B4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="83">
   <si>
     <t>TC_ID</t>
   </si>
@@ -119,9 +119,6 @@
     <t>Please select trip dates</t>
   </si>
   <si>
-    <t>2 Traveller(s)</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -278,16 +275,16 @@
     <t>Test Data8</t>
   </si>
   <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
     <t>FAIL</t>
   </si>
   <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>17</t>
+    <t>2 members</t>
   </si>
 </sst>
 </file>
@@ -714,7 +711,7 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -744,24 +741,24 @@
         <v>12</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>4</v>
@@ -775,15 +772,15 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s" s="0">
         <v>6</v>
@@ -795,15 +792,15 @@
         <v>7</v>
       </c>
       <c r="M3" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s" s="0">
         <v>8</v>
@@ -815,21 +812,21 @@
         <v>7</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="M4" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s" s="0">
         <v>13</v>
@@ -841,10 +838,10 @@
         <v>7</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>14</v>
@@ -853,18 +850,18 @@
         <v>15</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="M5" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s" s="0">
         <v>16</v>
@@ -876,10 +873,10 @@
         <v>7</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>14</v>
@@ -888,15 +885,15 @@
         <v>15</v>
       </c>
       <c r="M6" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s" s="0">
         <v>17</v>
@@ -908,10 +905,10 @@
         <v>7</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>14</v>
@@ -920,21 +917,21 @@
         <v>15</v>
       </c>
       <c r="J7" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K7" t="s" s="0">
         <v>18</v>
       </c>
       <c r="M7" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s" s="0">
         <v>19</v>
@@ -946,10 +943,10 @@
         <v>7</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>14</v>
@@ -958,21 +955,21 @@
         <v>15</v>
       </c>
       <c r="J8" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K8" t="s" s="0">
         <v>18</v>
       </c>
       <c r="M8" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s" s="0">
         <v>20</v>
@@ -984,10 +981,10 @@
         <v>7</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>14</v>
@@ -996,21 +993,21 @@
         <v>15</v>
       </c>
       <c r="J9" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K9" t="s" s="0">
         <v>18</v>
       </c>
       <c r="M9" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>21</v>
@@ -1022,36 +1019,36 @@
         <v>7</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="H10" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I10" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="J10" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K10" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L10" t="s" s="0">
         <v>22</v>
       </c>
       <c r="M10" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s" s="0">
         <v>23</v>
@@ -1063,15 +1060,15 @@
         <v>24</v>
       </c>
       <c r="M11" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>25</v>
@@ -1083,10 +1080,10 @@
         <v>7</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G12" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>14</v>
@@ -1095,232 +1092,232 @@
         <v>15</v>
       </c>
       <c r="J12" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K12" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L12" t="s" s="0">
         <v>26</v>
       </c>
       <c r="M12" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D13" t="s" s="0">
         <v>4</v>
       </c>
       <c r="M13" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D14" t="s" s="0">
         <v>4</v>
       </c>
       <c r="F14" s="2"/>
       <c r="M14" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E15" t="s" s="0">
         <v>46</v>
-      </c>
-      <c r="D15" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="E15" t="s" s="0">
-        <v>47</v>
       </c>
       <c r="F15" s="2"/>
       <c r="M15" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D16" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="E16" t="s" s="0">
-        <v>47</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="M16" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G17" t="s" s="0">
         <v>50</v>
       </c>
-      <c r="D17" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="E17" t="s" s="0">
-        <v>47</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G17" t="s" s="0">
-        <v>51</v>
-      </c>
       <c r="M17" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G18" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="H18" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="D18" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>47</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G18" t="s" s="0">
-        <v>51</v>
-      </c>
-      <c r="H18" t="s" s="0">
-        <v>53</v>
-      </c>
       <c r="M18" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C19" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G19" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="H19" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="I19" t="s" s="0">
         <v>54</v>
       </c>
-      <c r="D19" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="E19" t="s" s="0">
-        <v>47</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G19" t="s" s="0">
-        <v>51</v>
-      </c>
-      <c r="H19" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="I19" t="s" s="0">
-        <v>55</v>
-      </c>
       <c r="M19" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s" s="0">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G20" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="H20" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="I20" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="J20" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="D20" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>47</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G20" t="s" s="0">
-        <v>51</v>
-      </c>
-      <c r="H20" t="s" s="0">
-        <v>53</v>
-      </c>
-      <c r="I20" t="s" s="0">
-        <v>55</v>
-      </c>
-      <c r="J20" t="s" s="0">
+      <c r="K20" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s" s="0">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D21" t="s" s="0">
         <v>4</v>
@@ -1329,18 +1326,18 @@
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
       <c r="M21" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s" s="0">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D22" t="s" s="0">
         <v>4</v>
@@ -1349,44 +1346,44 @@
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
       <c r="M22" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s" s="0">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>69</v>
-      </c>
       <c r="M23" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s" s="0">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D24" t="s" s="0">
         <v>4</v>
       </c>
       <c r="M24" t="s" s="0">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Smoke and Regression Suite Added
</commit_message>
<xml_diff>
--- a/testdata/Scenario1_2_3_TestData.xlsx
+++ b/testdata/Scenario1_2_3_TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2408439\CTS_Java_Training\Practicals\IntelliJ_Selenium_Projects\Hackathon_Project\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F16A5436-00B7-401A-AC8E-AEADEA46929A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F833DC-5FE7-4C26-B948-329F3D8D3345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DE57E9C9-A6C1-4A7D-85B9-1309751074B4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="83">
   <si>
     <t>TC_ID</t>
   </si>
@@ -282,6 +282,9 @@
   </si>
   <si>
     <t>23</t>
+  </si>
+  <si>
+    <t>25</t>
   </si>
 </sst>
 </file>
@@ -809,10 +812,10 @@
         <v>7</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="M4" t="s" s="0">
         <v>69</v>
@@ -835,10 +838,10 @@
         <v>7</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>14</v>
@@ -870,10 +873,10 @@
         <v>7</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>14</v>
@@ -902,10 +905,10 @@
         <v>7</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>14</v>
@@ -940,10 +943,10 @@
         <v>7</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>14</v>
@@ -978,10 +981,10 @@
         <v>7</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>14</v>
@@ -1016,10 +1019,10 @@
         <v>7</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="H10" t="s" s="0">
         <v>79</v>

</xml_diff>